<commit_message>
"v1.7.3. Update xlsx wiring"
</commit_message>
<xml_diff>
--- a/docs/wiring.xlsx
+++ b/docs/wiring.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\01-home\14-python\gitTrackedCode\spiClock\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E932DD-C07E-4560-A473-347FC5E1A25F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD06DA7B-0F28-49E7-8A1E-7CC86F5FC519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2790" yWindow="0" windowWidth="21600" windowHeight="15585" xr2:uid="{BBCFC7B8-5D04-41D4-8F46-6DA2F5E1E523}"/>
+    <workbookView xWindow="4035" yWindow="675" windowWidth="22890" windowHeight="13500" activeTab="1" xr2:uid="{BBCFC7B8-5D04-41D4-8F46-6DA2F5E1E523}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="orig" sheetId="2" r:id="rId1"/>
+    <sheet name="split" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="49">
   <si>
     <t>vcc</t>
   </si>
@@ -246,7 +247,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -640,11 +641,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
@@ -698,6 +725,25 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -725,28 +771,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -781,10 +818,10 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="36" name="Straight Connector 35">
+        <xdr:cNvPr id="2" name="Straight Connector 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D29E1277-A7CA-6216-A777-D7377AACC253}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D77AD129-B69C-429A-BCB8-4504DC76568D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -792,8 +829,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5294586" y="3185948"/>
-          <a:ext cx="0" cy="394138"/>
+          <a:off x="5270609" y="5855247"/>
+          <a:ext cx="0" cy="361950"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -831,10 +868,10 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="37" name="Straight Connector 36">
+        <xdr:cNvPr id="3" name="Straight Connector 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{600D2627-D74A-4BFA-B969-30A90CAF220C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{215A503B-7FCD-463B-8712-161775E60F75}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -842,8 +879,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5098831" y="3187262"/>
-          <a:ext cx="0" cy="394138"/>
+          <a:off x="5075511" y="5856561"/>
+          <a:ext cx="0" cy="361950"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -881,10 +918,10 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="38" name="Straight Connector 37">
+        <xdr:cNvPr id="4" name="Straight Connector 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5E259CA-95C6-4BB9-B7FF-23D12BEA8D3B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A79EAFF-0C56-4F5F-B5B7-95977D5C0E7E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -892,8 +929,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4469524" y="3162299"/>
-          <a:ext cx="0" cy="394138"/>
+          <a:off x="4448175" y="5831598"/>
+          <a:ext cx="0" cy="361950"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -931,10 +968,10 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="39" name="Straight Connector 38">
+        <xdr:cNvPr id="5" name="Straight Connector 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B95ACBB4-8E2B-4448-BCC8-6741A1CE6170}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71C2612E-D91F-4CB0-B545-0C6096D2A1A5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -942,8 +979,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4687613" y="3163613"/>
-          <a:ext cx="0" cy="394138"/>
+          <a:off x="4665607" y="5832912"/>
+          <a:ext cx="0" cy="361950"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -981,10 +1018,10 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="40" name="Straight Connector 39">
+        <xdr:cNvPr id="6" name="Straight Connector 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D531D8C-C772-4777-9AFA-A12821909D0D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25596513-C311-4FD3-98B6-1902121C9509}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -992,8 +1029,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4242238" y="3164927"/>
-          <a:ext cx="0" cy="394138"/>
+          <a:off x="4221546" y="5834226"/>
+          <a:ext cx="0" cy="361950"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -1031,10 +1068,10 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="41" name="Straight Connector 40">
+        <xdr:cNvPr id="7" name="Straight Connector 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62AE4C7E-8CC5-4C40-AC21-520D571932F1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A16789C6-95A7-4CF4-BF11-6DC62D1ACA83}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1042,8 +1079,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3829707" y="3185948"/>
-          <a:ext cx="0" cy="394138"/>
+          <a:off x="3810329" y="5855247"/>
+          <a:ext cx="0" cy="361950"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -1081,6 +1118,1011 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="8" name="Straight Connector 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{468FD1A9-BD57-4E52-B3B6-307046FA5905}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3595522" y="5863129"/>
+          <a:ext cx="0" cy="361950"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>112985</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>112985</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>80134</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="9" name="Straight Connector 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{182B348E-EACF-4926-B519-FBB436CDBFAE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5285060" y="4533900"/>
+          <a:ext cx="0" cy="584959"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>127437</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>127437</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>81448</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="10" name="Straight Connector 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F9D45DC-800D-45AF-ACC2-9A37B3B55CB0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5089962" y="4514850"/>
+          <a:ext cx="0" cy="605323"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>128751</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>128751</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="11" name="Straight Connector 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3DA7220-6FC4-45B7-84F0-AA9D6ABE4137}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4462626" y="4533900"/>
+          <a:ext cx="0" cy="619125"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>136633</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>136633</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="12" name="Straight Connector 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{679EC95F-8FC4-40FA-AA1D-9B2237D2778A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4680058" y="4524375"/>
+          <a:ext cx="0" cy="609600"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>111672</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>111672</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="13" name="Straight Connector 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43A175A6-7F36-47DA-810D-1C9F09C22648}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4235997" y="4524375"/>
+          <a:ext cx="0" cy="600075"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>119555</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>119555</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>80134</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="14" name="Straight Connector 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6DDCB0DE-45C9-40FA-9DBA-811089C97570}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3824780" y="4514850"/>
+          <a:ext cx="0" cy="604009"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>114298</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>114298</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>88016</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="15" name="Straight Connector 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79452457-8C73-419F-9088-736534351922}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3609973" y="4514850"/>
+          <a:ext cx="0" cy="611891"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>116918</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>116918</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>116919</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="16" name="Straight Connector 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46DFB87A-0F39-4495-87A9-0B59DAC8A9AD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2983943" y="4514850"/>
+          <a:ext cx="0" cy="640794"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>124800</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>124800</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>118233</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="17" name="Straight Connector 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A88CDDB1-7B0D-48B3-AF88-09682AC84B20}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3201375" y="4524375"/>
+          <a:ext cx="0" cy="632583"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>99839</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>99839</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>119547</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="18" name="Straight Connector 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75CEA2E8-85CC-4D82-A57D-28BA1ACF1FC4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2757314" y="4524375"/>
+          <a:ext cx="0" cy="633897"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>118228</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>118228</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>105094</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="19" name="Straight Connector 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81AC2B6F-4110-4902-A81E-7716AED7D5C9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2356603" y="4524375"/>
+          <a:ext cx="0" cy="619444"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>126110</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>126110</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>106408</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="20" name="Straight Connector 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6EF39050-DF24-4E14-922E-FAC5B01EED05}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2574035" y="4524375"/>
+          <a:ext cx="0" cy="620758"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>101149</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>101149</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>107722</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="21" name="Straight Connector 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ABA84012-80A3-4D9B-9AC0-37FED10D62B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2129974" y="4533900"/>
+          <a:ext cx="0" cy="612547"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>111672</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>98534</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>4329</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="36" name="Straight Connector 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D29E1277-A7CA-6216-A777-D7377AACC253}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="5247409" y="5874297"/>
+          <a:ext cx="3284" cy="247680"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>112986</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>112986</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>112986</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>8659</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="37" name="Straight Connector 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{600D2627-D74A-4BFA-B969-30A90CAF220C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5057327" y="5875611"/>
+          <a:ext cx="0" cy="423878"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>88023</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="38" name="Straight Connector 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5E259CA-95C6-4BB9-B7FF-23D12BEA8D3B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4435186" y="5850648"/>
+          <a:ext cx="0" cy="786545"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>122182</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>89337</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>122182</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>4330</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="39" name="Straight Connector 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B95ACBB4-8E2B-4448-BCC8-6741A1CE6170}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4650887" y="5851962"/>
+          <a:ext cx="0" cy="616379"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>97221</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>90651</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>97221</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="40" name="Straight Connector 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D531D8C-C772-4777-9AFA-A12821909D0D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4210289" y="5853276"/>
+          <a:ext cx="0" cy="957099"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>105104</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>111672</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>105104</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>4329</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="41" name="Straight Connector 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62AE4C7E-8CC5-4C40-AC21-520D571932F1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3802536" y="5874297"/>
+          <a:ext cx="0" cy="1113589"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>99847</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>119554</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
         <xdr:cNvPr id="42" name="Straight Connector 41">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
@@ -1092,8 +2134,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3614244" y="3193830"/>
-          <a:ext cx="0" cy="394138"/>
+          <a:off x="3595522" y="5863129"/>
+          <a:ext cx="4928" cy="1271096"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -1744,6 +2786,706 @@
         <a:xfrm>
           <a:off x="920299" y="1781175"/>
           <a:ext cx="0" cy="669697"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="13" name="Straight Connector 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB30CA97-D2A2-4714-A0D5-DA4E9FA0E310}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3590925" y="7115175"/>
+          <a:ext cx="5295900" cy="28575"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="16" name="Straight Connector 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B72E1AA-61B4-45AA-861A-0803CA80EBEF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3800475" y="6972300"/>
+          <a:ext cx="5295900" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="18" name="Straight Connector 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D924C94-7A4A-475A-9559-8BF106C18695}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4210050" y="6781800"/>
+          <a:ext cx="5295900" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="19" name="Straight Connector 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{737C8814-EBA9-483F-A3CA-74EDF16C1ACA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4438650" y="6619875"/>
+          <a:ext cx="5295900" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="20" name="Straight Connector 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B867CE2E-F26C-4784-B272-EF55E7432A8C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4657725" y="6448425"/>
+          <a:ext cx="5295900" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>44</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="21" name="Straight Connector 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC76D308-1BA9-4F96-A468-241C6D1A0587}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5067300" y="6276975"/>
+          <a:ext cx="5295900" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="22" name="Straight Connector 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B0C9720-F4A7-498B-A4B9-5DE5D7912287}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5267325" y="6115050"/>
+          <a:ext cx="5295900" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>113434</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>130722</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>116718</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>23379</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="23" name="Straight Connector 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E89F622B-BC18-4FB7-8C2E-0B7CE891FC2F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="10562359" y="5874297"/>
+          <a:ext cx="3284" cy="245082"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>44</xdr:col>
+      <xdr:colOff>103461</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>122511</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>44</xdr:col>
+      <xdr:colOff>103461</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>18184</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="24" name="Straight Connector 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E19BDE1F-54FD-43B7-A8B5-724F704A31F4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10342836" y="5866086"/>
+          <a:ext cx="0" cy="419548"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>97548</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="25" name="Straight Connector 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DA86523-3844-4E57-8832-7E6896489D0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9715500" y="5841123"/>
+          <a:ext cx="0" cy="778752"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>112657</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>98862</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>112657</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>13855</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="26" name="Straight Connector 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6C8BD51-5856-4A90-8633-FCFF2058F31E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9932932" y="5842437"/>
+          <a:ext cx="0" cy="610318"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>87696</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>100176</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>87696</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="27" name="Straight Connector 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B4239C1-905B-4835-9C58-664BD0916464}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9488871" y="5843751"/>
+          <a:ext cx="0" cy="947574"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>95579</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>121197</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>95579</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>13854</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="28" name="Straight Connector 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5122BA5C-304F-4537-8438-1F7D1ED042F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9077654" y="5864772"/>
+          <a:ext cx="0" cy="1102332"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>90322</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>129079</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="29" name="Straight Connector 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0F350A2-A900-4F8B-A624-7273C53E3909}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8862847" y="5872654"/>
+          <a:ext cx="4928" cy="1271096"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -2085,7 +3827,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF5EE95F-D272-490C-AA41-F0BE02A6886D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A045644F-06CD-4953-8FEE-006E14B97CC9}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
@@ -2107,70 +3849,70 @@
   <sheetData>
     <row r="1" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B2" s="53"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
-      <c r="Q2" s="54"/>
-      <c r="R2" s="54"/>
-      <c r="S2" s="54"/>
-      <c r="T2" s="54"/>
-      <c r="U2" s="54"/>
-      <c r="V2" s="54"/>
-      <c r="W2" s="54"/>
-      <c r="X2" s="54"/>
-      <c r="Y2" s="54"/>
-      <c r="Z2" s="54"/>
-      <c r="AA2" s="54"/>
-      <c r="AB2" s="54"/>
-      <c r="AC2" s="54"/>
-      <c r="AD2" s="55"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="43"/>
+      <c r="V2" s="43"/>
+      <c r="W2" s="43"/>
+      <c r="X2" s="43"/>
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="43"/>
+      <c r="AA2" s="43"/>
+      <c r="AB2" s="43"/>
+      <c r="AC2" s="43"/>
+      <c r="AD2" s="44"/>
     </row>
     <row r="3" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="56"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57"/>
-      <c r="L3" s="57"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="57"/>
-      <c r="W3" s="57"/>
-      <c r="X3" s="57"/>
-      <c r="Y3" s="57"/>
-      <c r="Z3" s="57"/>
-      <c r="AA3" s="57"/>
-      <c r="AB3" s="57"/>
-      <c r="AC3" s="57"/>
-      <c r="AD3" s="58"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="46"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="46"/>
+      <c r="R3" s="46"/>
+      <c r="S3" s="46"/>
+      <c r="T3" s="46"/>
+      <c r="U3" s="46"/>
+      <c r="V3" s="46"/>
+      <c r="W3" s="46"/>
+      <c r="X3" s="46"/>
+      <c r="Y3" s="46"/>
+      <c r="Z3" s="46"/>
+      <c r="AA3" s="46"/>
+      <c r="AB3" s="46"/>
+      <c r="AC3" s="46"/>
+      <c r="AD3" s="47"/>
     </row>
     <row r="4" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="56"/>
-      <c r="C4" s="57"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="46"/>
       <c r="D4" s="26"/>
       <c r="E4" s="27"/>
       <c r="F4" s="27"/>
@@ -2194,210 +3936,109 @@
       <c r="X4" s="27"/>
       <c r="Y4" s="27"/>
       <c r="Z4" s="28"/>
-      <c r="AA4" s="57"/>
-      <c r="AB4" s="57"/>
-      <c r="AC4" s="57"/>
-      <c r="AD4" s="58"/>
+      <c r="AA4" s="46"/>
+      <c r="AB4" s="46"/>
+      <c r="AC4" s="46"/>
+      <c r="AD4" s="47"/>
     </row>
     <row r="5" spans="2:30" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="56"/>
-      <c r="C5" s="57"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
       <c r="D5" s="29"/>
-      <c r="E5" s="45" t="s">
+      <c r="E5" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="46"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-      <c r="L5" s="51" t="s">
+      <c r="F5" s="59"/>
+      <c r="G5" s="60"/>
+      <c r="L5" s="61" t="s">
         <v>47</v>
       </c>
-      <c r="M5" s="51"/>
-      <c r="N5" s="51"/>
-      <c r="O5" s="51"/>
-      <c r="P5" s="51"/>
-      <c r="Q5" s="51"/>
-      <c r="R5" s="51"/>
-      <c r="S5" s="49"/>
-      <c r="T5" s="49"/>
-      <c r="U5" s="49"/>
-      <c r="V5" s="49"/>
-      <c r="W5" s="49"/>
-      <c r="X5" s="49"/>
-      <c r="Y5" s="49"/>
+      <c r="M5" s="61"/>
+      <c r="N5" s="61"/>
+      <c r="O5" s="61"/>
+      <c r="P5" s="61"/>
+      <c r="Q5" s="61"/>
+      <c r="R5" s="61"/>
       <c r="Z5" s="30"/>
-      <c r="AA5" s="57"/>
-      <c r="AB5" s="57"/>
-      <c r="AC5" s="57"/>
-      <c r="AD5" s="58"/>
+      <c r="AA5" s="46"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="46"/>
+      <c r="AD5" s="47"/>
     </row>
     <row r="6" spans="2:30" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="56"/>
-      <c r="C6" s="57"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="46"/>
       <c r="D6" s="29"/>
-      <c r="E6" s="45" t="s">
+      <c r="E6" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="46"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="51"/>
-      <c r="O6" s="51"/>
-      <c r="P6" s="51"/>
-      <c r="Q6" s="51"/>
-      <c r="R6" s="51"/>
-      <c r="S6" s="49"/>
-      <c r="T6" s="49"/>
-      <c r="U6" s="49"/>
-      <c r="V6" s="49"/>
-      <c r="W6" s="49"/>
-      <c r="X6" s="49"/>
-      <c r="Y6" s="49"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="60"/>
+      <c r="L6" s="61"/>
+      <c r="M6" s="61"/>
+      <c r="N6" s="61"/>
+      <c r="O6" s="61"/>
+      <c r="P6" s="61"/>
+      <c r="Q6" s="61"/>
+      <c r="R6" s="61"/>
       <c r="Z6" s="30"/>
-      <c r="AA6" s="57"/>
-      <c r="AB6" s="57"/>
-      <c r="AC6" s="57"/>
-      <c r="AD6" s="58"/>
+      <c r="AA6" s="46"/>
+      <c r="AB6" s="46"/>
+      <c r="AC6" s="46"/>
+      <c r="AD6" s="47"/>
     </row>
     <row r="7" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="56"/>
-      <c r="C7" s="57"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="46"/>
       <c r="D7" s="29"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="49"/>
-      <c r="L7" s="49"/>
-      <c r="M7" s="49"/>
-      <c r="N7" s="49"/>
-      <c r="O7" s="49"/>
-      <c r="P7" s="49"/>
-      <c r="Q7" s="49"/>
-      <c r="R7" s="49"/>
-      <c r="S7" s="49"/>
-      <c r="T7" s="49"/>
-      <c r="U7" s="49"/>
-      <c r="V7" s="49"/>
-      <c r="W7" s="49"/>
-      <c r="X7" s="49"/>
-      <c r="Y7" s="49"/>
       <c r="Z7" s="30"/>
-      <c r="AA7" s="57"/>
-      <c r="AB7" s="57"/>
-      <c r="AC7" s="57"/>
-      <c r="AD7" s="58"/>
+      <c r="AA7" s="46"/>
+      <c r="AB7" s="46"/>
+      <c r="AC7" s="46"/>
+      <c r="AD7" s="47"/>
     </row>
     <row r="8" spans="2:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="56"/>
-      <c r="C8" s="57"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="46"/>
       <c r="D8" s="29"/>
-      <c r="E8" s="39" t="s">
+      <c r="E8" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="40"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="49"/>
-      <c r="I8" s="49"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="49"/>
-      <c r="L8" s="49"/>
-      <c r="M8" s="49"/>
-      <c r="N8" s="49"/>
-      <c r="O8" s="49"/>
-      <c r="P8" s="49"/>
-      <c r="Q8" s="49"/>
-      <c r="R8" s="49"/>
-      <c r="S8" s="49"/>
-      <c r="T8" s="49"/>
-      <c r="U8" s="49"/>
-      <c r="V8" s="49"/>
-      <c r="W8" s="49"/>
-      <c r="X8" s="49"/>
-      <c r="Y8" s="49"/>
+      <c r="F8" s="53"/>
+      <c r="G8" s="54"/>
       <c r="Z8" s="30"/>
-      <c r="AA8" s="57"/>
-      <c r="AB8" s="57"/>
-      <c r="AC8" s="57"/>
-      <c r="AD8" s="58"/>
+      <c r="AA8" s="46"/>
+      <c r="AB8" s="46"/>
+      <c r="AC8" s="46"/>
+      <c r="AD8" s="47"/>
     </row>
     <row r="9" spans="2:30" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="56"/>
-      <c r="C9" s="57"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="46"/>
       <c r="D9" s="29"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="49"/>
-      <c r="N9" s="49"/>
-      <c r="O9" s="49"/>
-      <c r="P9" s="49"/>
-      <c r="Q9" s="49"/>
-      <c r="R9" s="49"/>
-      <c r="S9" s="49"/>
-      <c r="T9" s="49"/>
-      <c r="U9" s="49"/>
-      <c r="V9" s="49"/>
-      <c r="W9" s="49"/>
-      <c r="X9" s="49"/>
-      <c r="Y9" s="49"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="57"/>
       <c r="Z9" s="30"/>
-      <c r="AA9" s="57"/>
-      <c r="AB9" s="57"/>
-      <c r="AC9" s="57"/>
-      <c r="AD9" s="58"/>
+      <c r="AA9" s="46"/>
+      <c r="AB9" s="46"/>
+      <c r="AC9" s="46"/>
+      <c r="AD9" s="47"/>
     </row>
     <row r="10" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B10" s="56"/>
-      <c r="C10" s="57"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="46"/>
       <c r="D10" s="29"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="49"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="49"/>
-      <c r="L10" s="49"/>
-      <c r="M10" s="49"/>
-      <c r="N10" s="49"/>
-      <c r="O10" s="49"/>
-      <c r="P10" s="49"/>
-      <c r="Q10" s="49"/>
-      <c r="R10" s="49"/>
-      <c r="S10" s="49"/>
-      <c r="T10" s="49"/>
-      <c r="U10" s="49"/>
-      <c r="V10" s="49"/>
-      <c r="W10" s="49"/>
-      <c r="X10" s="49"/>
-      <c r="Y10" s="49"/>
       <c r="Z10" s="30"/>
-      <c r="AA10" s="57"/>
-      <c r="AB10" s="57"/>
-      <c r="AC10" s="57"/>
-      <c r="AD10" s="58"/>
+      <c r="AA10" s="46"/>
+      <c r="AB10" s="46"/>
+      <c r="AC10" s="46"/>
+      <c r="AD10" s="47"/>
     </row>
     <row r="11" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B11" s="56"/>
-      <c r="C11" s="57"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="46"/>
       <c r="D11" s="29"/>
-      <c r="E11" s="49"/>
       <c r="F11" s="15">
         <v>39</v>
       </c>
@@ -2459,16 +4100,15 @@
         <v>1</v>
       </c>
       <c r="Z11" s="30"/>
-      <c r="AA11" s="57"/>
-      <c r="AB11" s="57"/>
-      <c r="AC11" s="57"/>
-      <c r="AD11" s="58"/>
+      <c r="AA11" s="46"/>
+      <c r="AB11" s="46"/>
+      <c r="AC11" s="46"/>
+      <c r="AD11" s="47"/>
     </row>
     <row r="12" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B12" s="56"/>
-      <c r="C12" s="57"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="46"/>
       <c r="D12" s="29"/>
-      <c r="E12" s="49"/>
       <c r="F12" s="15">
         <v>40</v>
       </c>
@@ -2530,14 +4170,14 @@
         <v>2</v>
       </c>
       <c r="Z12" s="30"/>
-      <c r="AA12" s="57"/>
-      <c r="AB12" s="57"/>
-      <c r="AC12" s="57"/>
-      <c r="AD12" s="58"/>
+      <c r="AA12" s="46"/>
+      <c r="AB12" s="46"/>
+      <c r="AC12" s="46"/>
+      <c r="AD12" s="47"/>
     </row>
     <row r="13" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="56"/>
-      <c r="C13" s="57"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="46"/>
       <c r="D13" s="31"/>
       <c r="E13" s="32"/>
       <c r="F13" s="32"/>
@@ -2561,45 +4201,45 @@
       <c r="X13" s="32"/>
       <c r="Y13" s="32"/>
       <c r="Z13" s="33"/>
-      <c r="AA13" s="57"/>
-      <c r="AB13" s="57"/>
-      <c r="AC13" s="57"/>
-      <c r="AD13" s="58"/>
+      <c r="AA13" s="46"/>
+      <c r="AB13" s="46"/>
+      <c r="AC13" s="46"/>
+      <c r="AD13" s="47"/>
     </row>
     <row r="14" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="56"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
-      <c r="G14" s="57"/>
-      <c r="H14" s="57"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="57"/>
-      <c r="K14" s="57"/>
-      <c r="L14" s="57"/>
-      <c r="M14" s="57"/>
-      <c r="N14" s="57"/>
-      <c r="O14" s="57"/>
-      <c r="P14" s="57"/>
-      <c r="Q14" s="57"/>
-      <c r="R14" s="57"/>
-      <c r="S14" s="57"/>
-      <c r="T14" s="57"/>
-      <c r="U14" s="57"/>
-      <c r="V14" s="57"/>
-      <c r="W14" s="57"/>
-      <c r="X14" s="57"/>
-      <c r="Y14" s="57"/>
-      <c r="Z14" s="57"/>
-      <c r="AA14" s="57"/>
-      <c r="AB14" s="57"/>
-      <c r="AC14" s="57"/>
-      <c r="AD14" s="58"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46"/>
+      <c r="K14" s="46"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="46"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="46"/>
+      <c r="U14" s="46"/>
+      <c r="V14" s="46"/>
+      <c r="W14" s="46"/>
+      <c r="X14" s="46"/>
+      <c r="Y14" s="46"/>
+      <c r="Z14" s="46"/>
+      <c r="AA14" s="46"/>
+      <c r="AB14" s="46"/>
+      <c r="AC14" s="46"/>
+      <c r="AD14" s="47"/>
     </row>
     <row r="15" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="56"/>
-      <c r="C15" s="57"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="46"/>
       <c r="D15" s="26"/>
       <c r="E15" s="27"/>
       <c r="F15" s="27"/>
@@ -2626,17 +4266,12 @@
       <c r="AA15" s="27"/>
       <c r="AB15" s="27"/>
       <c r="AC15" s="28"/>
-      <c r="AD15" s="58"/>
+      <c r="AD15" s="47"/>
     </row>
     <row r="16" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="56"/>
-      <c r="C16" s="57"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="46"/>
       <c r="D16" s="29"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="49"/>
-      <c r="I16" s="49"/>
       <c r="J16" s="37">
         <v>29</v>
       </c>
@@ -2682,20 +4317,13 @@
       <c r="Z16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AA16" s="49"/>
-      <c r="AB16" s="49"/>
       <c r="AC16" s="30"/>
-      <c r="AD16" s="58"/>
+      <c r="AD16" s="47"/>
     </row>
     <row r="17" spans="2:30" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="56"/>
-      <c r="C17" s="57"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="46"/>
       <c r="D17" s="29"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="49"/>
       <c r="J17" s="4" t="s">
         <v>42</v>
       </c>
@@ -2741,20 +4369,13 @@
       <c r="Z17" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="AA17" s="49"/>
-      <c r="AB17" s="49"/>
       <c r="AC17" s="30"/>
-      <c r="AD17" s="58"/>
+      <c r="AD17" s="47"/>
     </row>
     <row r="18" spans="2:30" ht="42.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="56"/>
-      <c r="C18" s="57"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="46"/>
       <c r="D18" s="29"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="49"/>
-      <c r="G18" s="49"/>
-      <c r="H18" s="49"/>
-      <c r="I18" s="49"/>
       <c r="J18" s="4" t="s">
         <v>18</v>
       </c>
@@ -2800,112 +4421,49 @@
       <c r="Z18" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="AA18" s="49"/>
-      <c r="AB18" s="49"/>
       <c r="AC18" s="30"/>
-      <c r="AD18" s="58"/>
+      <c r="AD18" s="47"/>
     </row>
     <row r="19" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B19" s="56"/>
-      <c r="C19" s="57"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="46"/>
       <c r="D19" s="29"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="49"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="48"/>
-      <c r="K19" s="48"/>
-      <c r="L19" s="48"/>
-      <c r="M19" s="48"/>
-      <c r="N19" s="48"/>
-      <c r="O19" s="48"/>
-      <c r="P19" s="48"/>
-      <c r="Q19" s="48"/>
-      <c r="R19" s="48"/>
-      <c r="S19" s="48"/>
-      <c r="T19" s="48"/>
-      <c r="U19" s="48"/>
-      <c r="V19" s="48"/>
-      <c r="W19" s="49"/>
-      <c r="X19" s="48"/>
-      <c r="Y19" s="48"/>
-      <c r="Z19" s="49"/>
-      <c r="AA19" s="49"/>
-      <c r="AB19" s="49"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="39"/>
+      <c r="L19" s="39"/>
+      <c r="M19" s="39"/>
+      <c r="N19" s="39"/>
+      <c r="O19" s="39"/>
+      <c r="P19" s="39"/>
+      <c r="Q19" s="39"/>
+      <c r="R19" s="39"/>
+      <c r="S19" s="39"/>
+      <c r="T19" s="39"/>
+      <c r="U19" s="39"/>
+      <c r="V19" s="39"/>
+      <c r="X19" s="39"/>
+      <c r="Y19" s="39"/>
       <c r="AC19" s="30"/>
-      <c r="AD19" s="58"/>
+      <c r="AD19" s="47"/>
     </row>
     <row r="20" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B20" s="56"/>
-      <c r="C20" s="57"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="46"/>
       <c r="D20" s="29"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="49"/>
-      <c r="I20" s="49"/>
-      <c r="J20" s="49"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="49"/>
-      <c r="M20" s="49"/>
-      <c r="N20" s="49"/>
-      <c r="O20" s="49"/>
-      <c r="P20" s="49"/>
-      <c r="Q20" s="49"/>
-      <c r="R20" s="49"/>
-      <c r="S20" s="49"/>
-      <c r="T20" s="49"/>
-      <c r="U20" s="49"/>
-      <c r="V20" s="49"/>
-      <c r="W20" s="49"/>
-      <c r="X20" s="49"/>
-      <c r="Y20" s="49"/>
-      <c r="Z20" s="49"/>
-      <c r="AA20" s="49"/>
-      <c r="AB20" s="49"/>
       <c r="AC20" s="30"/>
-      <c r="AD20" s="58"/>
+      <c r="AD20" s="47"/>
     </row>
     <row r="21" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="56"/>
-      <c r="C21" s="57"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="46"/>
       <c r="D21" s="29"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="49"/>
-      <c r="I21" s="49"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="49"/>
-      <c r="N21" s="49"/>
-      <c r="O21" s="49"/>
-      <c r="P21" s="49"/>
-      <c r="Q21" s="49"/>
-      <c r="R21" s="49"/>
-      <c r="S21" s="49"/>
-      <c r="T21" s="49"/>
-      <c r="U21" s="49"/>
-      <c r="V21" s="49"/>
-      <c r="W21" s="49"/>
-      <c r="X21" s="49"/>
-      <c r="Y21" s="49"/>
-      <c r="Z21" s="49"/>
-      <c r="AA21" s="49"/>
-      <c r="AB21" s="49"/>
       <c r="AC21" s="30"/>
-      <c r="AD21" s="58"/>
+      <c r="AD21" s="47"/>
     </row>
     <row r="22" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="56"/>
-      <c r="C22" s="57"/>
+      <c r="B22" s="45"/>
+      <c r="C22" s="46"/>
       <c r="D22" s="29"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="49"/>
-      <c r="H22" s="49"/>
       <c r="I22" s="9"/>
       <c r="J22" s="10"/>
       <c r="K22" s="10"/>
@@ -2923,7 +4481,6 @@
       <c r="W22" s="9"/>
       <c r="X22" s="10"/>
       <c r="Y22" s="11"/>
-      <c r="Z22" s="49"/>
       <c r="AA22" s="12" t="s">
         <v>20</v>
       </c>
@@ -2931,16 +4488,12 @@
         <v>21</v>
       </c>
       <c r="AC22" s="30"/>
-      <c r="AD22" s="58"/>
+      <c r="AD22" s="47"/>
     </row>
     <row r="23" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B23" s="56"/>
-      <c r="C23" s="57"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="46"/>
       <c r="D23" s="29"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
       <c r="I23" s="14"/>
       <c r="J23" s="15"/>
       <c r="K23" s="15"/>
@@ -2958,7 +4511,6 @@
       <c r="W23" s="14"/>
       <c r="X23" s="15"/>
       <c r="Y23" s="16"/>
-      <c r="Z23" s="49"/>
       <c r="AA23" s="17" t="s">
         <v>7</v>
       </c>
@@ -2966,16 +4518,12 @@
         <v>1</v>
       </c>
       <c r="AC23" s="30"/>
-      <c r="AD23" s="58"/>
+      <c r="AD23" s="47"/>
     </row>
     <row r="24" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B24" s="56"/>
-      <c r="C24" s="57"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="46"/>
       <c r="D24" s="29"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="49"/>
       <c r="I24" s="14"/>
       <c r="J24" s="15"/>
       <c r="K24" s="15"/>
@@ -2993,7 +4541,6 @@
       <c r="W24" s="14"/>
       <c r="X24" s="15"/>
       <c r="Y24" s="16"/>
-      <c r="Z24" s="49"/>
       <c r="AA24" s="19" t="s">
         <v>8</v>
       </c>
@@ -3001,16 +4548,12 @@
         <v>2</v>
       </c>
       <c r="AC24" s="30"/>
-      <c r="AD24" s="58"/>
+      <c r="AD24" s="47"/>
     </row>
     <row r="25" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="56"/>
-      <c r="C25" s="57"/>
+      <c r="B25" s="45"/>
+      <c r="C25" s="46"/>
       <c r="D25" s="29"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
       <c r="I25" s="14"/>
       <c r="J25" s="15"/>
       <c r="K25" s="15"/>
@@ -3028,7 +4571,6 @@
       <c r="W25" s="14"/>
       <c r="X25" s="15"/>
       <c r="Y25" s="16"/>
-      <c r="Z25" s="49"/>
       <c r="AA25" s="21" t="s">
         <v>9</v>
       </c>
@@ -3036,16 +4578,12 @@
         <v>3</v>
       </c>
       <c r="AC25" s="30"/>
-      <c r="AD25" s="58"/>
+      <c r="AD25" s="47"/>
     </row>
     <row r="26" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="56"/>
-      <c r="C26" s="57"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="46"/>
       <c r="D26" s="29"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="49"/>
       <c r="I26" s="23"/>
       <c r="J26" s="24"/>
       <c r="K26" s="24"/>
@@ -3063,51 +4601,22 @@
       <c r="W26" s="23"/>
       <c r="X26" s="24"/>
       <c r="Y26" s="25"/>
-      <c r="Z26" s="49"/>
-      <c r="AA26" s="49"/>
-      <c r="AB26" s="52"/>
+      <c r="AB26" s="41"/>
       <c r="AC26" s="30"/>
-      <c r="AD26" s="58"/>
+      <c r="AD26" s="47"/>
     </row>
     <row r="27" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="56"/>
-      <c r="C27" s="57"/>
+      <c r="B27" s="45"/>
+      <c r="C27" s="46"/>
       <c r="D27" s="29"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="49"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="49"/>
-      <c r="M27" s="49"/>
-      <c r="N27" s="49"/>
-      <c r="O27" s="49"/>
-      <c r="P27" s="49"/>
-      <c r="Q27" s="49"/>
-      <c r="R27" s="49"/>
-      <c r="S27" s="49"/>
-      <c r="T27" s="49"/>
-      <c r="U27" s="49"/>
-      <c r="V27" s="49"/>
-      <c r="W27" s="49"/>
-      <c r="X27" s="49"/>
-      <c r="Y27" s="49"/>
-      <c r="Z27" s="49"/>
-      <c r="AA27" s="49"/>
-      <c r="AB27" s="52"/>
+      <c r="AB27" s="41"/>
       <c r="AC27" s="30"/>
-      <c r="AD27" s="58"/>
+      <c r="AD27" s="47"/>
     </row>
     <row r="28" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="56"/>
-      <c r="C28" s="57"/>
+      <c r="B28" s="45"/>
+      <c r="C28" s="46"/>
       <c r="D28" s="29"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="49"/>
-      <c r="H28" s="49"/>
       <c r="I28" s="9"/>
       <c r="J28" s="9"/>
       <c r="K28" s="9"/>
@@ -3125,7 +4634,6 @@
       <c r="W28" s="9"/>
       <c r="X28" s="10"/>
       <c r="Y28" s="11"/>
-      <c r="Z28" s="49"/>
       <c r="AA28" s="12" t="s">
         <v>20</v>
       </c>
@@ -3133,16 +4641,12 @@
         <v>21</v>
       </c>
       <c r="AC28" s="30"/>
-      <c r="AD28" s="58"/>
+      <c r="AD28" s="47"/>
     </row>
     <row r="29" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B29" s="56"/>
-      <c r="C29" s="57"/>
+      <c r="B29" s="45"/>
+      <c r="C29" s="46"/>
       <c r="D29" s="29"/>
-      <c r="E29" s="49"/>
-      <c r="F29" s="49"/>
-      <c r="G29" s="49"/>
-      <c r="H29" s="49"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14"/>
       <c r="K29" s="14"/>
@@ -3160,7 +4664,6 @@
       <c r="W29" s="14"/>
       <c r="X29" s="15"/>
       <c r="Y29" s="16"/>
-      <c r="Z29" s="49"/>
       <c r="AA29" s="17" t="s">
         <v>10</v>
       </c>
@@ -3168,16 +4671,12 @@
         <v>4</v>
       </c>
       <c r="AC29" s="30"/>
-      <c r="AD29" s="58"/>
+      <c r="AD29" s="47"/>
     </row>
     <row r="30" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B30" s="56"/>
-      <c r="C30" s="57"/>
+      <c r="B30" s="45"/>
+      <c r="C30" s="46"/>
       <c r="D30" s="29"/>
-      <c r="E30" s="49"/>
-      <c r="F30" s="49"/>
-      <c r="G30" s="49"/>
-      <c r="H30" s="49"/>
       <c r="I30" s="14"/>
       <c r="J30" s="14"/>
       <c r="K30" s="14"/>
@@ -3195,7 +4694,6 @@
       <c r="W30" s="14"/>
       <c r="X30" s="15"/>
       <c r="Y30" s="16"/>
-      <c r="Z30" s="49"/>
       <c r="AA30" s="19" t="s">
         <v>11</v>
       </c>
@@ -3203,16 +4701,12 @@
         <v>5</v>
       </c>
       <c r="AC30" s="30"/>
-      <c r="AD30" s="58"/>
+      <c r="AD30" s="47"/>
     </row>
     <row r="31" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="56"/>
-      <c r="C31" s="57"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="46"/>
       <c r="D31" s="29"/>
-      <c r="E31" s="49"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="49"/>
-      <c r="H31" s="49"/>
       <c r="I31" s="14"/>
       <c r="J31" s="14"/>
       <c r="K31" s="14"/>
@@ -3230,7 +4724,6 @@
       <c r="W31" s="14"/>
       <c r="X31" s="15"/>
       <c r="Y31" s="16"/>
-      <c r="Z31" s="49"/>
       <c r="AA31" s="21" t="s">
         <v>12</v>
       </c>
@@ -3238,16 +4731,12 @@
         <v>6</v>
       </c>
       <c r="AC31" s="30"/>
-      <c r="AD31" s="58"/>
+      <c r="AD31" s="47"/>
     </row>
     <row r="32" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="56"/>
-      <c r="C32" s="57"/>
+      <c r="B32" s="45"/>
+      <c r="C32" s="46"/>
       <c r="D32" s="29"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="49"/>
-      <c r="H32" s="49"/>
       <c r="I32" s="23"/>
       <c r="J32" s="23"/>
       <c r="K32" s="23"/>
@@ -3265,52 +4754,20 @@
       <c r="W32" s="23"/>
       <c r="X32" s="24"/>
       <c r="Y32" s="25"/>
-      <c r="Z32" s="49"/>
-      <c r="AA32" s="49"/>
-      <c r="AB32" s="49"/>
       <c r="AC32" s="30"/>
-      <c r="AD32" s="58"/>
+      <c r="AD32" s="47"/>
     </row>
     <row r="33" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="56"/>
-      <c r="C33" s="57"/>
+      <c r="B33" s="45"/>
+      <c r="C33" s="46"/>
       <c r="D33" s="29"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="49"/>
-      <c r="L33" s="49"/>
-      <c r="M33" s="49"/>
-      <c r="N33" s="49"/>
-      <c r="O33" s="49"/>
-      <c r="P33" s="49"/>
-      <c r="Q33" s="49"/>
-      <c r="R33" s="49"/>
-      <c r="S33" s="49"/>
-      <c r="T33" s="49"/>
-      <c r="U33" s="49"/>
-      <c r="V33" s="49"/>
-      <c r="W33" s="49"/>
-      <c r="X33" s="49"/>
-      <c r="Y33" s="49"/>
-      <c r="Z33" s="49"/>
-      <c r="AA33" s="49"/>
-      <c r="AB33" s="49"/>
       <c r="AC33" s="30"/>
-      <c r="AD33" s="58"/>
+      <c r="AD33" s="47"/>
     </row>
     <row r="34" spans="2:30" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="56"/>
-      <c r="C34" s="57"/>
+      <c r="B34" s="45"/>
+      <c r="C34" s="46"/>
       <c r="D34" s="29"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="49"/>
-      <c r="H34" s="49"/>
-      <c r="I34" s="49"/>
       <c r="J34" s="4" t="s">
         <v>29</v>
       </c>
@@ -3356,78 +4813,61 @@
       <c r="Z34" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AA34" s="49"/>
-      <c r="AB34" s="49"/>
       <c r="AC34" s="30"/>
-      <c r="AD34" s="58"/>
+      <c r="AD34" s="47"/>
     </row>
     <row r="35" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B35" s="56"/>
-      <c r="C35" s="57"/>
+      <c r="B35" s="45"/>
+      <c r="C35" s="46"/>
       <c r="D35" s="29"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="49"/>
-      <c r="I35" s="49"/>
-      <c r="J35" s="48"/>
-      <c r="K35" s="48"/>
-      <c r="L35" s="48"/>
-      <c r="M35" s="48"/>
-      <c r="N35" s="48"/>
-      <c r="O35" s="48"/>
-      <c r="P35" s="48"/>
-      <c r="Q35" s="48"/>
-      <c r="R35" s="48"/>
-      <c r="S35" s="48"/>
-      <c r="T35" s="48"/>
-      <c r="U35" s="48"/>
-      <c r="V35" s="48"/>
-      <c r="W35" s="49"/>
-      <c r="X35" s="48"/>
-      <c r="Y35" s="48"/>
-      <c r="Z35" s="50"/>
-      <c r="AA35" s="49"/>
-      <c r="AB35" s="49"/>
+      <c r="J35" s="39"/>
+      <c r="K35" s="39"/>
+      <c r="L35" s="39"/>
+      <c r="M35" s="39"/>
+      <c r="N35" s="39"/>
+      <c r="O35" s="39"/>
+      <c r="P35" s="39"/>
+      <c r="Q35" s="39"/>
+      <c r="R35" s="39"/>
+      <c r="S35" s="39"/>
+      <c r="T35" s="39"/>
+      <c r="U35" s="39"/>
+      <c r="V35" s="39"/>
+      <c r="X35" s="39"/>
+      <c r="Y35" s="39"/>
+      <c r="Z35" s="40"/>
       <c r="AC35" s="30"/>
-      <c r="AD35" s="58"/>
+      <c r="AD35" s="47"/>
     </row>
     <row r="36" spans="2:30" ht="24.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="56"/>
-      <c r="C36" s="57"/>
+      <c r="B36" s="45"/>
+      <c r="C36" s="46"/>
       <c r="D36" s="29"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="49"/>
-      <c r="G36" s="49"/>
-      <c r="H36" s="49"/>
-      <c r="I36" s="49"/>
-      <c r="J36" s="51" t="s">
+      <c r="J36" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="K36" s="51"/>
-      <c r="L36" s="51"/>
-      <c r="M36" s="51"/>
-      <c r="N36" s="51"/>
-      <c r="O36" s="51"/>
-      <c r="P36" s="51"/>
-      <c r="Q36" s="51"/>
-      <c r="R36" s="51"/>
-      <c r="S36" s="51"/>
-      <c r="T36" s="51"/>
-      <c r="U36" s="51"/>
-      <c r="V36" s="51"/>
-      <c r="W36" s="51"/>
-      <c r="X36" s="51"/>
-      <c r="Y36" s="51"/>
-      <c r="Z36" s="50"/>
-      <c r="AA36" s="49"/>
-      <c r="AB36" s="49"/>
+      <c r="K36" s="61"/>
+      <c r="L36" s="61"/>
+      <c r="M36" s="61"/>
+      <c r="N36" s="61"/>
+      <c r="O36" s="61"/>
+      <c r="P36" s="61"/>
+      <c r="Q36" s="61"/>
+      <c r="R36" s="61"/>
+      <c r="S36" s="61"/>
+      <c r="T36" s="61"/>
+      <c r="U36" s="61"/>
+      <c r="V36" s="61"/>
+      <c r="W36" s="61"/>
+      <c r="X36" s="61"/>
+      <c r="Y36" s="61"/>
+      <c r="Z36" s="40"/>
       <c r="AC36" s="30"/>
-      <c r="AD36" s="58"/>
+      <c r="AD36" s="47"/>
     </row>
     <row r="37" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="56"/>
-      <c r="C37" s="57"/>
+      <c r="B37" s="45"/>
+      <c r="C37" s="46"/>
       <c r="D37" s="31"/>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
@@ -3454,38 +4894,1518 @@
       <c r="AA37" s="32"/>
       <c r="AB37" s="32"/>
       <c r="AC37" s="33"/>
-      <c r="AD37" s="58"/>
+      <c r="AD37" s="47"/>
     </row>
     <row r="38" spans="2:30" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="59"/>
-      <c r="C38" s="60"/>
-      <c r="D38" s="60"/>
-      <c r="E38" s="60"/>
-      <c r="F38" s="60"/>
-      <c r="G38" s="60"/>
-      <c r="H38" s="60"/>
-      <c r="I38" s="60"/>
-      <c r="J38" s="60"/>
-      <c r="K38" s="60"/>
-      <c r="L38" s="60"/>
-      <c r="M38" s="60"/>
-      <c r="N38" s="60"/>
-      <c r="O38" s="60"/>
-      <c r="P38" s="60"/>
-      <c r="Q38" s="60"/>
-      <c r="R38" s="60"/>
-      <c r="S38" s="60"/>
-      <c r="T38" s="60"/>
-      <c r="U38" s="60"/>
-      <c r="V38" s="60"/>
-      <c r="W38" s="60"/>
-      <c r="X38" s="60"/>
-      <c r="Y38" s="60"/>
-      <c r="Z38" s="60"/>
-      <c r="AA38" s="60"/>
-      <c r="AB38" s="60"/>
-      <c r="AC38" s="60"/>
-      <c r="AD38" s="61"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="49"/>
+      <c r="D38" s="49"/>
+      <c r="E38" s="49"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
+      <c r="I38" s="49"/>
+      <c r="J38" s="49"/>
+      <c r="K38" s="49"/>
+      <c r="L38" s="49"/>
+      <c r="M38" s="49"/>
+      <c r="N38" s="49"/>
+      <c r="O38" s="49"/>
+      <c r="P38" s="49"/>
+      <c r="Q38" s="49"/>
+      <c r="R38" s="49"/>
+      <c r="S38" s="49"/>
+      <c r="T38" s="49"/>
+      <c r="U38" s="49"/>
+      <c r="V38" s="49"/>
+      <c r="W38" s="49"/>
+      <c r="X38" s="49"/>
+      <c r="Y38" s="49"/>
+      <c r="Z38" s="49"/>
+      <c r="AA38" s="49"/>
+      <c r="AB38" s="49"/>
+      <c r="AC38" s="49"/>
+      <c r="AD38" s="50"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="L5:R6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="E8:G9"/>
+    <mergeCell ref="J36:Y36"/>
+  </mergeCells>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup scale="97" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF5EE95F-D272-490C-AA41-F0BE02A6886D}">
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:AY38"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="3.140625" style="1" customWidth="1"/>
+    <col min="4" max="8" width="3.28515625" style="1" customWidth="1"/>
+    <col min="9" max="25" width="3.140625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="6.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="2.7109375" style="1" customWidth="1"/>
+    <col min="30" max="47" width="3.140625" style="1" customWidth="1"/>
+    <col min="48" max="48" width="7.85546875" style="1" customWidth="1"/>
+    <col min="49" max="49" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="3.140625" style="1" customWidth="1"/>
+    <col min="51" max="51" width="5" style="1" customWidth="1"/>
+    <col min="52" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B2" s="42"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="43"/>
+      <c r="V2" s="43"/>
+      <c r="W2" s="43"/>
+      <c r="X2" s="43"/>
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="43"/>
+      <c r="AA2" s="43"/>
+      <c r="AB2" s="43"/>
+      <c r="AC2" s="43"/>
+      <c r="AD2" s="43"/>
+      <c r="AE2" s="43"/>
+      <c r="AF2" s="43"/>
+      <c r="AG2" s="43"/>
+      <c r="AH2" s="43"/>
+      <c r="AI2" s="43"/>
+      <c r="AJ2" s="43"/>
+      <c r="AK2" s="43"/>
+      <c r="AL2" s="43"/>
+      <c r="AM2" s="43"/>
+      <c r="AN2" s="43"/>
+      <c r="AO2" s="43"/>
+      <c r="AP2" s="43"/>
+      <c r="AQ2" s="43"/>
+      <c r="AR2" s="43"/>
+      <c r="AS2" s="43"/>
+      <c r="AT2" s="43"/>
+      <c r="AU2" s="43"/>
+      <c r="AV2" s="43"/>
+      <c r="AW2" s="43"/>
+      <c r="AX2" s="43"/>
+      <c r="AY2" s="44"/>
+    </row>
+    <row r="3" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="45"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="46"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="46"/>
+      <c r="R3" s="46"/>
+      <c r="S3" s="46"/>
+      <c r="T3" s="46"/>
+      <c r="U3" s="46"/>
+      <c r="V3" s="46"/>
+      <c r="W3" s="46"/>
+      <c r="X3" s="46"/>
+      <c r="Y3" s="46"/>
+      <c r="Z3" s="46"/>
+      <c r="AA3" s="46"/>
+      <c r="AB3" s="46"/>
+      <c r="AC3" s="46"/>
+      <c r="AD3" s="46"/>
+      <c r="AE3" s="46"/>
+      <c r="AF3" s="46"/>
+      <c r="AG3" s="46"/>
+      <c r="AH3" s="46"/>
+      <c r="AI3" s="46"/>
+      <c r="AJ3" s="46"/>
+      <c r="AK3" s="46"/>
+      <c r="AL3" s="46"/>
+      <c r="AM3" s="46"/>
+      <c r="AN3" s="46"/>
+      <c r="AO3" s="46"/>
+      <c r="AP3" s="46"/>
+      <c r="AQ3" s="46"/>
+      <c r="AR3" s="46"/>
+      <c r="AS3" s="46"/>
+      <c r="AT3" s="46"/>
+      <c r="AU3" s="46"/>
+      <c r="AV3" s="46"/>
+      <c r="AW3" s="46"/>
+      <c r="AX3" s="46"/>
+      <c r="AY3" s="47"/>
+    </row>
+    <row r="4" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="45"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="27"/>
+      <c r="S4" s="27"/>
+      <c r="T4" s="27"/>
+      <c r="U4" s="27"/>
+      <c r="V4" s="27"/>
+      <c r="W4" s="27"/>
+      <c r="X4" s="27"/>
+      <c r="Y4" s="27"/>
+      <c r="Z4" s="28"/>
+      <c r="AA4" s="46"/>
+      <c r="AB4" s="46"/>
+      <c r="AC4" s="46"/>
+      <c r="AD4" s="46"/>
+      <c r="AE4" s="46"/>
+      <c r="AF4" s="46"/>
+      <c r="AG4" s="46"/>
+      <c r="AH4" s="46"/>
+      <c r="AI4" s="46"/>
+      <c r="AJ4" s="46"/>
+      <c r="AK4" s="46"/>
+      <c r="AL4" s="46"/>
+      <c r="AM4" s="46"/>
+      <c r="AN4" s="46"/>
+      <c r="AO4" s="46"/>
+      <c r="AP4" s="46"/>
+      <c r="AQ4" s="46"/>
+      <c r="AR4" s="46"/>
+      <c r="AS4" s="46"/>
+      <c r="AT4" s="46"/>
+      <c r="AU4" s="46"/>
+      <c r="AV4" s="46"/>
+      <c r="AW4" s="46"/>
+      <c r="AX4" s="46"/>
+      <c r="AY4" s="47"/>
+    </row>
+    <row r="5" spans="2:51" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="59"/>
+      <c r="G5" s="60"/>
+      <c r="L5" s="61" t="s">
+        <v>47</v>
+      </c>
+      <c r="M5" s="61"/>
+      <c r="N5" s="61"/>
+      <c r="O5" s="61"/>
+      <c r="P5" s="61"/>
+      <c r="Q5" s="61"/>
+      <c r="R5" s="61"/>
+      <c r="Z5" s="30"/>
+      <c r="AA5" s="46"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="46"/>
+      <c r="AD5" s="46"/>
+      <c r="AE5" s="46"/>
+      <c r="AF5" s="46"/>
+      <c r="AG5" s="46"/>
+      <c r="AH5" s="46"/>
+      <c r="AI5" s="46"/>
+      <c r="AJ5" s="46"/>
+      <c r="AK5" s="46"/>
+      <c r="AL5" s="46"/>
+      <c r="AM5" s="46"/>
+      <c r="AN5" s="46"/>
+      <c r="AO5" s="46"/>
+      <c r="AP5" s="46"/>
+      <c r="AQ5" s="46"/>
+      <c r="AR5" s="46"/>
+      <c r="AS5" s="46"/>
+      <c r="AT5" s="46"/>
+      <c r="AU5" s="46"/>
+      <c r="AV5" s="46"/>
+      <c r="AW5" s="46"/>
+      <c r="AX5" s="46"/>
+      <c r="AY5" s="47"/>
+    </row>
+    <row r="6" spans="2:51" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="45"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="58" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="59"/>
+      <c r="G6" s="60"/>
+      <c r="L6" s="61"/>
+      <c r="M6" s="61"/>
+      <c r="N6" s="61"/>
+      <c r="O6" s="61"/>
+      <c r="P6" s="61"/>
+      <c r="Q6" s="61"/>
+      <c r="R6" s="61"/>
+      <c r="Z6" s="30"/>
+      <c r="AA6" s="46"/>
+      <c r="AB6" s="46"/>
+      <c r="AC6" s="46"/>
+      <c r="AD6" s="46"/>
+      <c r="AE6" s="46"/>
+      <c r="AF6" s="46"/>
+      <c r="AG6" s="46"/>
+      <c r="AH6" s="46"/>
+      <c r="AI6" s="46"/>
+      <c r="AJ6" s="46"/>
+      <c r="AK6" s="46"/>
+      <c r="AL6" s="46"/>
+      <c r="AM6" s="46"/>
+      <c r="AN6" s="46"/>
+      <c r="AO6" s="46"/>
+      <c r="AP6" s="46"/>
+      <c r="AQ6" s="46"/>
+      <c r="AR6" s="46"/>
+      <c r="AS6" s="46"/>
+      <c r="AT6" s="46"/>
+      <c r="AU6" s="46"/>
+      <c r="AV6" s="46"/>
+      <c r="AW6" s="46"/>
+      <c r="AX6" s="46"/>
+      <c r="AY6" s="47"/>
+    </row>
+    <row r="7" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="45"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="29"/>
+      <c r="Z7" s="30"/>
+      <c r="AA7" s="46"/>
+      <c r="AB7" s="46"/>
+      <c r="AC7" s="46"/>
+      <c r="AD7" s="46"/>
+      <c r="AE7" s="46"/>
+      <c r="AF7" s="46"/>
+      <c r="AG7" s="46"/>
+      <c r="AH7" s="46"/>
+      <c r="AI7" s="46"/>
+      <c r="AJ7" s="46"/>
+      <c r="AK7" s="46"/>
+      <c r="AL7" s="46"/>
+      <c r="AM7" s="46"/>
+      <c r="AN7" s="46"/>
+      <c r="AO7" s="46"/>
+      <c r="AP7" s="46"/>
+      <c r="AQ7" s="46"/>
+      <c r="AR7" s="46"/>
+      <c r="AS7" s="46"/>
+      <c r="AT7" s="46"/>
+      <c r="AU7" s="46"/>
+      <c r="AV7" s="46"/>
+      <c r="AW7" s="46"/>
+      <c r="AX7" s="46"/>
+      <c r="AY7" s="47"/>
+    </row>
+    <row r="8" spans="2:51" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="45"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="52" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="53"/>
+      <c r="G8" s="54"/>
+      <c r="Z8" s="30"/>
+      <c r="AA8" s="46"/>
+      <c r="AB8" s="46"/>
+      <c r="AC8" s="46"/>
+      <c r="AD8" s="46"/>
+      <c r="AE8" s="46"/>
+      <c r="AF8" s="46"/>
+      <c r="AG8" s="46"/>
+      <c r="AH8" s="46"/>
+      <c r="AI8" s="46"/>
+      <c r="AJ8" s="46"/>
+      <c r="AK8" s="46"/>
+      <c r="AL8" s="46"/>
+      <c r="AM8" s="46"/>
+      <c r="AN8" s="46"/>
+      <c r="AO8" s="46"/>
+      <c r="AP8" s="46"/>
+      <c r="AQ8" s="46"/>
+      <c r="AR8" s="46"/>
+      <c r="AS8" s="46"/>
+      <c r="AT8" s="46"/>
+      <c r="AU8" s="46"/>
+      <c r="AV8" s="46"/>
+      <c r="AW8" s="46"/>
+      <c r="AX8" s="46"/>
+      <c r="AY8" s="47"/>
+    </row>
+    <row r="9" spans="2:51" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="45"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="57"/>
+      <c r="Z9" s="30"/>
+      <c r="AA9" s="46"/>
+      <c r="AB9" s="46"/>
+      <c r="AC9" s="46"/>
+      <c r="AD9" s="46"/>
+      <c r="AE9" s="46"/>
+      <c r="AF9" s="46"/>
+      <c r="AG9" s="46"/>
+      <c r="AH9" s="46"/>
+      <c r="AI9" s="46"/>
+      <c r="AJ9" s="46"/>
+      <c r="AK9" s="46"/>
+      <c r="AL9" s="46"/>
+      <c r="AM9" s="46"/>
+      <c r="AN9" s="46"/>
+      <c r="AO9" s="46"/>
+      <c r="AP9" s="46"/>
+      <c r="AQ9" s="46"/>
+      <c r="AR9" s="46"/>
+      <c r="AS9" s="46"/>
+      <c r="AT9" s="46"/>
+      <c r="AU9" s="46"/>
+      <c r="AV9" s="46"/>
+      <c r="AW9" s="46"/>
+      <c r="AX9" s="46"/>
+      <c r="AY9" s="47"/>
+    </row>
+    <row r="10" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B10" s="45"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="29"/>
+      <c r="Z10" s="30"/>
+      <c r="AA10" s="46"/>
+      <c r="AB10" s="46"/>
+      <c r="AC10" s="46"/>
+      <c r="AD10" s="46"/>
+      <c r="AE10" s="46"/>
+      <c r="AF10" s="46"/>
+      <c r="AG10" s="46"/>
+      <c r="AH10" s="46"/>
+      <c r="AI10" s="46"/>
+      <c r="AJ10" s="46"/>
+      <c r="AK10" s="46"/>
+      <c r="AL10" s="46"/>
+      <c r="AM10" s="46"/>
+      <c r="AN10" s="46"/>
+      <c r="AO10" s="46"/>
+      <c r="AP10" s="46"/>
+      <c r="AQ10" s="46"/>
+      <c r="AR10" s="46"/>
+      <c r="AS10" s="46"/>
+      <c r="AT10" s="46"/>
+      <c r="AU10" s="46"/>
+      <c r="AV10" s="46"/>
+      <c r="AW10" s="46"/>
+      <c r="AX10" s="46"/>
+      <c r="AY10" s="47"/>
+    </row>
+    <row r="11" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B11" s="45"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="29"/>
+      <c r="F11" s="15">
+        <v>39</v>
+      </c>
+      <c r="G11" s="34">
+        <v>37</v>
+      </c>
+      <c r="H11" s="15">
+        <v>35</v>
+      </c>
+      <c r="I11" s="15">
+        <v>33</v>
+      </c>
+      <c r="J11" s="34">
+        <v>31</v>
+      </c>
+      <c r="K11" s="34">
+        <v>29</v>
+      </c>
+      <c r="L11" s="15">
+        <v>27</v>
+      </c>
+      <c r="M11" s="15">
+        <v>25</v>
+      </c>
+      <c r="N11" s="14">
+        <v>23</v>
+      </c>
+      <c r="O11" s="15">
+        <v>21</v>
+      </c>
+      <c r="P11" s="14">
+        <v>19</v>
+      </c>
+      <c r="Q11" s="15">
+        <v>17</v>
+      </c>
+      <c r="R11" s="34">
+        <v>15</v>
+      </c>
+      <c r="S11" s="14">
+        <v>13</v>
+      </c>
+      <c r="T11" s="34">
+        <v>11</v>
+      </c>
+      <c r="U11" s="15">
+        <v>9</v>
+      </c>
+      <c r="V11" s="15">
+        <v>7</v>
+      </c>
+      <c r="W11" s="15">
+        <v>5</v>
+      </c>
+      <c r="X11" s="15">
+        <v>3</v>
+      </c>
+      <c r="Y11" s="14">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="30"/>
+      <c r="AA11" s="46"/>
+      <c r="AB11" s="46"/>
+      <c r="AC11" s="46"/>
+      <c r="AD11" s="46"/>
+      <c r="AE11" s="46"/>
+      <c r="AF11" s="46"/>
+      <c r="AG11" s="46"/>
+      <c r="AH11" s="46"/>
+      <c r="AI11" s="46"/>
+      <c r="AJ11" s="46"/>
+      <c r="AK11" s="46"/>
+      <c r="AL11" s="46"/>
+      <c r="AM11" s="46"/>
+      <c r="AN11" s="46"/>
+      <c r="AO11" s="46"/>
+      <c r="AP11" s="46"/>
+      <c r="AQ11" s="46"/>
+      <c r="AR11" s="46"/>
+      <c r="AS11" s="46"/>
+      <c r="AT11" s="46"/>
+      <c r="AU11" s="46"/>
+      <c r="AV11" s="46"/>
+      <c r="AW11" s="46"/>
+      <c r="AX11" s="46"/>
+      <c r="AY11" s="47"/>
+    </row>
+    <row r="12" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B12" s="45"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="29"/>
+      <c r="F12" s="15">
+        <v>40</v>
+      </c>
+      <c r="G12" s="15">
+        <v>38</v>
+      </c>
+      <c r="H12" s="15">
+        <v>36</v>
+      </c>
+      <c r="I12" s="15">
+        <v>34</v>
+      </c>
+      <c r="J12" s="15">
+        <v>32</v>
+      </c>
+      <c r="K12" s="15">
+        <v>30</v>
+      </c>
+      <c r="L12" s="15">
+        <v>28</v>
+      </c>
+      <c r="M12" s="15">
+        <v>26</v>
+      </c>
+      <c r="N12" s="15">
+        <v>24</v>
+      </c>
+      <c r="O12" s="14">
+        <v>22</v>
+      </c>
+      <c r="P12" s="15">
+        <v>20</v>
+      </c>
+      <c r="Q12" s="15">
+        <v>18</v>
+      </c>
+      <c r="R12" s="34">
+        <v>16</v>
+      </c>
+      <c r="S12" s="15">
+        <v>14</v>
+      </c>
+      <c r="T12" s="14">
+        <v>12</v>
+      </c>
+      <c r="U12" s="15">
+        <v>10</v>
+      </c>
+      <c r="V12" s="15">
+        <v>8</v>
+      </c>
+      <c r="W12" s="14">
+        <v>6</v>
+      </c>
+      <c r="X12" s="15">
+        <v>4</v>
+      </c>
+      <c r="Y12" s="15">
+        <v>2</v>
+      </c>
+      <c r="Z12" s="30"/>
+      <c r="AA12" s="46"/>
+      <c r="AB12" s="46"/>
+      <c r="AC12" s="46"/>
+      <c r="AD12" s="46"/>
+      <c r="AE12" s="46"/>
+      <c r="AF12" s="46"/>
+      <c r="AG12" s="46"/>
+      <c r="AH12" s="46"/>
+      <c r="AI12" s="46"/>
+      <c r="AJ12" s="46"/>
+      <c r="AK12" s="46"/>
+      <c r="AL12" s="46"/>
+      <c r="AM12" s="46"/>
+      <c r="AN12" s="46"/>
+      <c r="AO12" s="46"/>
+      <c r="AP12" s="46"/>
+      <c r="AQ12" s="46"/>
+      <c r="AR12" s="46"/>
+      <c r="AS12" s="46"/>
+      <c r="AT12" s="46"/>
+      <c r="AU12" s="46"/>
+      <c r="AV12" s="46"/>
+      <c r="AW12" s="46"/>
+      <c r="AX12" s="46"/>
+      <c r="AY12" s="47"/>
+    </row>
+    <row r="13" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="45"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+      <c r="O13" s="32"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="32"/>
+      <c r="S13" s="32"/>
+      <c r="T13" s="32"/>
+      <c r="U13" s="32"/>
+      <c r="V13" s="32"/>
+      <c r="W13" s="32"/>
+      <c r="X13" s="32"/>
+      <c r="Y13" s="32"/>
+      <c r="Z13" s="33"/>
+      <c r="AA13" s="46"/>
+      <c r="AB13" s="46"/>
+      <c r="AC13" s="46"/>
+      <c r="AD13" s="46"/>
+      <c r="AE13" s="46"/>
+      <c r="AF13" s="46"/>
+      <c r="AG13" s="46"/>
+      <c r="AH13" s="46"/>
+      <c r="AI13" s="46"/>
+      <c r="AJ13" s="46"/>
+      <c r="AK13" s="46"/>
+      <c r="AL13" s="46"/>
+      <c r="AM13" s="46"/>
+      <c r="AN13" s="46"/>
+      <c r="AO13" s="46"/>
+      <c r="AP13" s="46"/>
+      <c r="AQ13" s="46"/>
+      <c r="AR13" s="46"/>
+      <c r="AS13" s="46"/>
+      <c r="AT13" s="46"/>
+      <c r="AU13" s="46"/>
+      <c r="AV13" s="46"/>
+      <c r="AW13" s="46"/>
+      <c r="AX13" s="46"/>
+      <c r="AY13" s="47"/>
+    </row>
+    <row r="14" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="45"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46"/>
+      <c r="K14" s="46"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="46"/>
+      <c r="S14" s="46"/>
+      <c r="T14" s="46"/>
+      <c r="U14" s="46"/>
+      <c r="V14" s="46"/>
+      <c r="W14" s="46"/>
+      <c r="X14" s="46"/>
+      <c r="Y14" s="46"/>
+      <c r="Z14" s="46"/>
+      <c r="AA14" s="46"/>
+      <c r="AB14" s="46"/>
+      <c r="AC14" s="46"/>
+      <c r="AD14" s="46"/>
+      <c r="AE14" s="46"/>
+      <c r="AF14" s="46"/>
+      <c r="AG14" s="46"/>
+      <c r="AH14" s="46"/>
+      <c r="AI14" s="46"/>
+      <c r="AJ14" s="46"/>
+      <c r="AK14" s="46"/>
+      <c r="AL14" s="46"/>
+      <c r="AM14" s="46"/>
+      <c r="AN14" s="46"/>
+      <c r="AO14" s="46"/>
+      <c r="AP14" s="46"/>
+      <c r="AQ14" s="46"/>
+      <c r="AR14" s="46"/>
+      <c r="AS14" s="46"/>
+      <c r="AT14" s="46"/>
+      <c r="AU14" s="46"/>
+      <c r="AV14" s="46"/>
+      <c r="AW14" s="46"/>
+      <c r="AX14" s="46"/>
+      <c r="AY14" s="47"/>
+    </row>
+    <row r="15" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="45"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="27"/>
+      <c r="R15" s="27"/>
+      <c r="S15" s="27"/>
+      <c r="T15" s="27"/>
+      <c r="U15" s="27"/>
+      <c r="V15" s="27"/>
+      <c r="W15" s="27"/>
+      <c r="X15" s="27"/>
+      <c r="Y15" s="27"/>
+      <c r="Z15" s="27"/>
+      <c r="AA15" s="27"/>
+      <c r="AB15" s="27"/>
+      <c r="AC15" s="27"/>
+      <c r="AD15" s="27"/>
+      <c r="AE15" s="27"/>
+      <c r="AF15" s="27"/>
+      <c r="AG15" s="27"/>
+      <c r="AH15" s="27"/>
+      <c r="AI15" s="27"/>
+      <c r="AJ15" s="27"/>
+      <c r="AK15" s="27"/>
+      <c r="AL15" s="27"/>
+      <c r="AM15" s="27"/>
+      <c r="AN15" s="27"/>
+      <c r="AO15" s="27"/>
+      <c r="AP15" s="27"/>
+      <c r="AQ15" s="27"/>
+      <c r="AR15" s="27"/>
+      <c r="AS15" s="27"/>
+      <c r="AT15" s="27"/>
+      <c r="AU15" s="27"/>
+      <c r="AV15" s="27"/>
+      <c r="AW15" s="27"/>
+      <c r="AX15" s="27"/>
+      <c r="AY15" s="51"/>
+    </row>
+    <row r="16" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="45"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="29"/>
+      <c r="J16" s="37">
+        <v>29</v>
+      </c>
+      <c r="K16" s="38">
+        <v>31</v>
+      </c>
+      <c r="L16" s="38">
+        <v>11</v>
+      </c>
+      <c r="M16" s="38">
+        <v>15</v>
+      </c>
+      <c r="N16" s="38">
+        <v>16</v>
+      </c>
+      <c r="O16" s="38">
+        <v>37</v>
+      </c>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="36">
+        <v>12</v>
+      </c>
+      <c r="R16" s="36">
+        <v>13</v>
+      </c>
+      <c r="S16" s="2"/>
+      <c r="T16" s="36">
+        <v>22</v>
+      </c>
+      <c r="U16" s="36">
+        <v>23</v>
+      </c>
+      <c r="V16" s="36">
+        <v>19</v>
+      </c>
+      <c r="W16" s="2"/>
+      <c r="X16" s="36">
+        <v>6</v>
+      </c>
+      <c r="Y16" s="35">
+        <v>1</v>
+      </c>
+      <c r="Z16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AY16" s="51"/>
+    </row>
+    <row r="17" spans="2:51" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="45"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="29"/>
+      <c r="J17" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S17" s="5"/>
+      <c r="T17" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="U17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="V17" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="W17" s="6"/>
+      <c r="X17" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="Z17" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="AY17" s="51"/>
+    </row>
+    <row r="18" spans="2:51" ht="42.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="45"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="29"/>
+      <c r="J18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="O18" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="R18" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="S18" s="5"/>
+      <c r="T18" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="U18" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="V18" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="W18" s="6"/>
+      <c r="X18" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y18" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="AY18" s="51"/>
+    </row>
+    <row r="19" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B19" s="45"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="29"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="39"/>
+      <c r="L19" s="39"/>
+      <c r="M19" s="39"/>
+      <c r="N19" s="39"/>
+      <c r="O19" s="39"/>
+      <c r="P19" s="39"/>
+      <c r="Q19" s="39"/>
+      <c r="R19" s="39"/>
+      <c r="S19" s="39"/>
+      <c r="T19" s="39"/>
+      <c r="U19" s="39"/>
+      <c r="V19" s="39"/>
+      <c r="X19" s="39"/>
+      <c r="Y19" s="39"/>
+      <c r="AY19" s="51"/>
+    </row>
+    <row r="20" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B20" s="45"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="29"/>
+      <c r="AY20" s="51"/>
+    </row>
+    <row r="21" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="45"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="29"/>
+      <c r="AY21" s="51"/>
+    </row>
+    <row r="22" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="45"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="29"/>
+      <c r="I22" s="65"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="10"/>
+      <c r="S22" s="9"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="10"/>
+      <c r="V22" s="10"/>
+      <c r="W22" s="9"/>
+      <c r="X22" s="10"/>
+      <c r="Y22" s="11"/>
+      <c r="AA22" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB22" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="AD22" s="65"/>
+      <c r="AE22" s="9"/>
+      <c r="AF22" s="9"/>
+      <c r="AG22" s="9"/>
+      <c r="AH22" s="9"/>
+      <c r="AI22" s="9"/>
+      <c r="AJ22" s="9"/>
+      <c r="AK22" s="9"/>
+      <c r="AL22" s="10"/>
+      <c r="AM22" s="10"/>
+      <c r="AN22" s="9"/>
+      <c r="AO22" s="10"/>
+      <c r="AP22" s="10"/>
+      <c r="AQ22" s="10"/>
+      <c r="AR22" s="9"/>
+      <c r="AS22" s="10"/>
+      <c r="AT22" s="11"/>
+      <c r="AV22" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="AW22" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="AY22" s="51"/>
+    </row>
+    <row r="23" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B23" s="45"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="29"/>
+      <c r="I23" s="66"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15"/>
+      <c r="L23" s="15"/>
+      <c r="M23" s="15"/>
+      <c r="N23" s="15"/>
+      <c r="O23" s="15"/>
+      <c r="P23" s="14"/>
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="14"/>
+      <c r="T23" s="15"/>
+      <c r="U23" s="15"/>
+      <c r="V23" s="15"/>
+      <c r="W23" s="14"/>
+      <c r="X23" s="15"/>
+      <c r="Y23" s="16"/>
+      <c r="AA23" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="AB23" s="18">
+        <v>1</v>
+      </c>
+      <c r="AD23" s="66"/>
+      <c r="AE23" s="14"/>
+      <c r="AF23" s="14"/>
+      <c r="AG23" s="14"/>
+      <c r="AH23" s="14"/>
+      <c r="AI23" s="14"/>
+      <c r="AJ23" s="14"/>
+      <c r="AK23" s="14"/>
+      <c r="AL23" s="15"/>
+      <c r="AM23" s="15"/>
+      <c r="AN23" s="14"/>
+      <c r="AO23" s="15"/>
+      <c r="AP23" s="15"/>
+      <c r="AQ23" s="15"/>
+      <c r="AR23" s="14"/>
+      <c r="AS23" s="15"/>
+      <c r="AT23" s="16"/>
+      <c r="AV23" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="AW23" s="18">
+        <v>4</v>
+      </c>
+      <c r="AY23" s="51"/>
+    </row>
+    <row r="24" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B24" s="45"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="29"/>
+      <c r="I24" s="66"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+      <c r="O24" s="15"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="15"/>
+      <c r="R24" s="15"/>
+      <c r="S24" s="14"/>
+      <c r="T24" s="15"/>
+      <c r="U24" s="15"/>
+      <c r="V24" s="15"/>
+      <c r="W24" s="14"/>
+      <c r="X24" s="15"/>
+      <c r="Y24" s="16"/>
+      <c r="AA24" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="AB24" s="20">
+        <v>2</v>
+      </c>
+      <c r="AD24" s="66"/>
+      <c r="AE24" s="14"/>
+      <c r="AF24" s="14"/>
+      <c r="AG24" s="14"/>
+      <c r="AH24" s="14"/>
+      <c r="AI24" s="14"/>
+      <c r="AJ24" s="14"/>
+      <c r="AK24" s="14"/>
+      <c r="AL24" s="15"/>
+      <c r="AM24" s="15"/>
+      <c r="AN24" s="14"/>
+      <c r="AO24" s="15"/>
+      <c r="AP24" s="15"/>
+      <c r="AQ24" s="15"/>
+      <c r="AR24" s="14"/>
+      <c r="AS24" s="15"/>
+      <c r="AT24" s="16"/>
+      <c r="AV24" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="AW24" s="20">
+        <v>5</v>
+      </c>
+      <c r="AY24" s="51"/>
+    </row>
+    <row r="25" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="45"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="29"/>
+      <c r="I25" s="66"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="15"/>
+      <c r="P25" s="14"/>
+      <c r="Q25" s="15"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="14"/>
+      <c r="T25" s="15"/>
+      <c r="U25" s="15"/>
+      <c r="V25" s="15"/>
+      <c r="W25" s="14"/>
+      <c r="X25" s="15"/>
+      <c r="Y25" s="16"/>
+      <c r="AA25" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB25" s="22">
+        <v>3</v>
+      </c>
+      <c r="AD25" s="66"/>
+      <c r="AE25" s="14"/>
+      <c r="AF25" s="14"/>
+      <c r="AG25" s="14"/>
+      <c r="AH25" s="14"/>
+      <c r="AI25" s="14"/>
+      <c r="AJ25" s="14"/>
+      <c r="AK25" s="14"/>
+      <c r="AL25" s="15"/>
+      <c r="AM25" s="15"/>
+      <c r="AN25" s="14"/>
+      <c r="AO25" s="15"/>
+      <c r="AP25" s="15"/>
+      <c r="AQ25" s="15"/>
+      <c r="AR25" s="14"/>
+      <c r="AS25" s="15"/>
+      <c r="AT25" s="16"/>
+      <c r="AV25" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="AW25" s="22">
+        <v>6</v>
+      </c>
+      <c r="AY25" s="51"/>
+    </row>
+    <row r="26" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="45"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="29"/>
+      <c r="I26" s="67"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24"/>
+      <c r="N26" s="24"/>
+      <c r="O26" s="24"/>
+      <c r="P26" s="23"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="24"/>
+      <c r="S26" s="23"/>
+      <c r="T26" s="24"/>
+      <c r="U26" s="24"/>
+      <c r="V26" s="24"/>
+      <c r="W26" s="23"/>
+      <c r="X26" s="24"/>
+      <c r="Y26" s="25"/>
+      <c r="AB26" s="41"/>
+      <c r="AD26" s="67"/>
+      <c r="AE26" s="23"/>
+      <c r="AF26" s="23"/>
+      <c r="AG26" s="23"/>
+      <c r="AH26" s="23"/>
+      <c r="AI26" s="23"/>
+      <c r="AJ26" s="23"/>
+      <c r="AK26" s="23"/>
+      <c r="AL26" s="24"/>
+      <c r="AM26" s="24"/>
+      <c r="AN26" s="23"/>
+      <c r="AO26" s="24"/>
+      <c r="AP26" s="24"/>
+      <c r="AQ26" s="24"/>
+      <c r="AR26" s="23"/>
+      <c r="AS26" s="24"/>
+      <c r="AT26" s="25"/>
+      <c r="AY26" s="51"/>
+    </row>
+    <row r="27" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B27" s="45"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="29"/>
+      <c r="AB27" s="41"/>
+      <c r="AY27" s="51"/>
+    </row>
+    <row r="28" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B28" s="45"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="29"/>
+      <c r="AY28" s="51"/>
+    </row>
+    <row r="29" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B29" s="45"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="29"/>
+      <c r="AY29" s="51"/>
+    </row>
+    <row r="30" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B30" s="45"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="29"/>
+      <c r="AY30" s="51"/>
+    </row>
+    <row r="31" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B31" s="45"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="29"/>
+      <c r="AY31" s="51"/>
+    </row>
+    <row r="32" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B32" s="45"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="29"/>
+      <c r="AY32" s="51"/>
+    </row>
+    <row r="33" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B33" s="45"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="29"/>
+      <c r="AY33" s="51"/>
+    </row>
+    <row r="34" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="45"/>
+      <c r="C34" s="46"/>
+      <c r="D34" s="29"/>
+      <c r="AY34" s="51"/>
+    </row>
+    <row r="35" spans="2:51" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="45"/>
+      <c r="C35" s="46"/>
+      <c r="D35" s="29"/>
+      <c r="J35" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="P35" s="5"/>
+      <c r="Q35" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="R35" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S35" s="5"/>
+      <c r="T35" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="U35" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="V35" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="W35" s="6"/>
+      <c r="X35" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z35" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD35" s="4"/>
+      <c r="AE35" s="5"/>
+      <c r="AF35" s="5"/>
+      <c r="AG35" s="5"/>
+      <c r="AH35" s="5"/>
+      <c r="AI35" s="5"/>
+      <c r="AJ35" s="5"/>
+      <c r="AK35" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AL35" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AM35" s="5"/>
+      <c r="AN35" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AO35" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AP35" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="AQ35" s="6"/>
+      <c r="AR35" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="AS35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="AT35" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AY35" s="51"/>
+    </row>
+    <row r="36" spans="2:51" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B36" s="45"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="K36" s="62"/>
+      <c r="L36" s="62"/>
+      <c r="M36" s="62"/>
+      <c r="N36" s="62"/>
+      <c r="O36" s="62"/>
+      <c r="P36" s="62"/>
+      <c r="Q36" s="62"/>
+      <c r="R36" s="62"/>
+      <c r="S36" s="62"/>
+      <c r="T36" s="62"/>
+      <c r="U36" s="62"/>
+      <c r="V36" s="62"/>
+      <c r="W36" s="62"/>
+      <c r="X36" s="62"/>
+      <c r="Y36" s="62"/>
+      <c r="Z36" s="62"/>
+      <c r="AA36" s="62"/>
+      <c r="AB36" s="62"/>
+      <c r="AC36" s="62"/>
+      <c r="AD36" s="62"/>
+      <c r="AE36" s="62"/>
+      <c r="AF36" s="62"/>
+      <c r="AG36" s="62"/>
+      <c r="AH36" s="62"/>
+      <c r="AI36" s="62"/>
+      <c r="AJ36" s="62"/>
+      <c r="AK36" s="62"/>
+      <c r="AL36" s="62"/>
+      <c r="AM36" s="62"/>
+      <c r="AN36" s="62"/>
+      <c r="AO36" s="62"/>
+      <c r="AP36" s="62"/>
+      <c r="AQ36" s="62"/>
+      <c r="AR36" s="62"/>
+      <c r="AS36" s="62"/>
+      <c r="AT36" s="62"/>
+      <c r="AU36" s="62"/>
+      <c r="AV36" s="62"/>
+      <c r="AW36" s="62"/>
+      <c r="AX36" s="64"/>
+      <c r="AY36" s="51"/>
+    </row>
+    <row r="37" spans="2:51" x14ac:dyDescent="0.25">
+      <c r="B37" s="45"/>
+      <c r="C37" s="46"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="63"/>
+      <c r="K37" s="63"/>
+      <c r="L37" s="63"/>
+      <c r="M37" s="63"/>
+      <c r="N37" s="63"/>
+      <c r="O37" s="63"/>
+      <c r="P37" s="63"/>
+      <c r="Q37" s="63"/>
+      <c r="R37" s="63"/>
+      <c r="S37" s="63"/>
+      <c r="T37" s="63"/>
+      <c r="U37" s="63"/>
+      <c r="V37" s="63"/>
+      <c r="W37" s="63"/>
+      <c r="X37" s="63"/>
+      <c r="Y37" s="63"/>
+      <c r="Z37" s="63"/>
+      <c r="AA37" s="63"/>
+      <c r="AB37" s="63"/>
+      <c r="AC37" s="63"/>
+      <c r="AD37" s="63"/>
+      <c r="AE37" s="63"/>
+      <c r="AF37" s="63"/>
+      <c r="AG37" s="63"/>
+      <c r="AH37" s="63"/>
+      <c r="AI37" s="63"/>
+      <c r="AJ37" s="63"/>
+      <c r="AK37" s="63"/>
+      <c r="AL37" s="63"/>
+      <c r="AM37" s="63"/>
+      <c r="AN37" s="63"/>
+      <c r="AO37" s="63"/>
+      <c r="AP37" s="63"/>
+      <c r="AQ37" s="63"/>
+      <c r="AR37" s="63"/>
+      <c r="AS37" s="63"/>
+      <c r="AT37" s="63"/>
+      <c r="AU37" s="63"/>
+      <c r="AV37" s="63"/>
+      <c r="AW37" s="63"/>
+      <c r="AX37" s="63"/>
+      <c r="AY37" s="47"/>
+    </row>
+    <row r="38" spans="2:51" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="48"/>
+      <c r="C38" s="49"/>
+      <c r="D38" s="49"/>
+      <c r="E38" s="49"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
+      <c r="I38" s="49"/>
+      <c r="J38" s="49"/>
+      <c r="K38" s="49"/>
+      <c r="L38" s="49"/>
+      <c r="M38" s="49"/>
+      <c r="N38" s="49"/>
+      <c r="O38" s="49"/>
+      <c r="P38" s="49"/>
+      <c r="Q38" s="49"/>
+      <c r="R38" s="49"/>
+      <c r="S38" s="49"/>
+      <c r="T38" s="49"/>
+      <c r="U38" s="49"/>
+      <c r="V38" s="49"/>
+      <c r="W38" s="49"/>
+      <c r="X38" s="49"/>
+      <c r="Y38" s="49"/>
+      <c r="Z38" s="49"/>
+      <c r="AA38" s="49"/>
+      <c r="AB38" s="49"/>
+      <c r="AC38" s="49"/>
+      <c r="AD38" s="49"/>
+      <c r="AE38" s="49"/>
+      <c r="AF38" s="49"/>
+      <c r="AG38" s="49"/>
+      <c r="AH38" s="49"/>
+      <c r="AI38" s="49"/>
+      <c r="AJ38" s="49"/>
+      <c r="AK38" s="49"/>
+      <c r="AL38" s="49"/>
+      <c r="AM38" s="49"/>
+      <c r="AN38" s="49"/>
+      <c r="AO38" s="49"/>
+      <c r="AP38" s="49"/>
+      <c r="AQ38" s="49"/>
+      <c r="AR38" s="49"/>
+      <c r="AS38" s="49"/>
+      <c r="AT38" s="49"/>
+      <c r="AU38" s="49"/>
+      <c r="AV38" s="49"/>
+      <c r="AW38" s="49"/>
+      <c r="AX38" s="49"/>
+      <c r="AY38" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3493,10 +6413,11 @@
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="E6:G6"/>
     <mergeCell ref="L5:R6"/>
-    <mergeCell ref="J36:Y36"/>
+    <mergeCell ref="J36:AX36"/>
   </mergeCells>
-  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup scale="97" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0"/>
+  <pageSetup scale="72" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>